<commit_message>
fix(settlements): correct June 2026 EoD pin (was ~2.8h early) (#156)
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/keel/2026-06/keel_settlement_june_2026.xlsx
+++ b/settlements/keel/2026-06/keel_settlement_june_2026.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Venues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Debt" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>32198.1297654743</v>
+        <v>30997.79005858496</v>
       </c>
     </row>
     <row r="6">
@@ -513,7 +513,7 @@
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>51769.8897654743</v>
+        <v>50569.55005858496</v>
       </c>
     </row>
     <row r="9">
@@ -612,7 +612,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ethereum=25433093</t>
+          <t>ethereum=25433938</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:56+00:00</t>
+          <t>2026-07-15T11:29:03+00:00</t>
         </is>
       </c>
     </row>
@@ -1069,10 +1069,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -1109,10 +1109,10 @@
         <v>0</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>0</v>
@@ -1149,10 +1149,10 @@
         <v>0</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>0</v>
@@ -1189,10 +1189,10 @@
         <v>0</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K9" s="3" t="n">
         <v>0</v>
@@ -1229,10 +1229,10 @@
         <v>0</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K10" s="3" t="n">
         <v>0</v>
@@ -1269,10 +1269,10 @@
         <v>0</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>0</v>
@@ -1309,10 +1309,10 @@
         <v>0</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>0</v>
@@ -1349,10 +1349,10 @@
         <v>0</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K13" s="3" t="n">
         <v>0</v>
@@ -1389,10 +1389,10 @@
         <v>0</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>0</v>
@@ -1429,10 +1429,10 @@
         <v>0</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J15" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K15" s="3" t="n">
         <v>0</v>
@@ -1469,10 +1469,10 @@
         <v>0</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J16" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>0</v>
@@ -1509,10 +1509,10 @@
         <v>0</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J17" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K17" s="3" t="n">
         <v>0</v>
@@ -1549,10 +1549,10 @@
         <v>0</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K18" s="3" t="n">
         <v>0</v>
@@ -1589,10 +1589,10 @@
         <v>0</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J19" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K19" s="3" t="n">
         <v>0</v>
@@ -1629,10 +1629,10 @@
         <v>0</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>0</v>
@@ -1669,10 +1669,10 @@
         <v>0</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K21" s="3" t="n">
         <v>0</v>
@@ -1709,10 +1709,10 @@
         <v>0</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K22" s="3" t="n">
         <v>0</v>
@@ -1749,10 +1749,10 @@
         <v>0</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K23" s="3" t="n">
         <v>0</v>
@@ -1789,10 +1789,10 @@
         <v>0</v>
       </c>
       <c r="I24" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J24" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K24" s="3" t="n">
         <v>0</v>
@@ -1829,10 +1829,10 @@
         <v>0</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J25" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K25" s="3" t="n">
         <v>0</v>
@@ -1869,10 +1869,10 @@
         <v>0</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K26" s="3" t="n">
         <v>0</v>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K27" s="3" t="n">
         <v>0</v>
@@ -1949,10 +1949,10 @@
         <v>0</v>
       </c>
       <c r="I28" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K28" s="3" t="n">
         <v>0</v>
@@ -1989,10 +1989,10 @@
         <v>0</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J29" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K29" s="3" t="n">
         <v>0</v>
@@ -2029,10 +2029,10 @@
         <v>0</v>
       </c>
       <c r="I30" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J30" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K30" s="3" t="n">
         <v>0</v>
@@ -2069,10 +2069,10 @@
         <v>0</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K31" s="3" t="n">
         <v>0</v>
@@ -2109,10 +2109,10 @@
         <v>0</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K32" s="3" t="n">
         <v>0</v>
@@ -2149,10 +2149,10 @@
         <v>0</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K33" s="3" t="n">
         <v>0</v>
@@ -2189,10 +2189,10 @@
         <v>0</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K34" s="3" t="n">
         <v>0</v>
@@ -2229,10 +2229,10 @@
         <v>0</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>0.03750000355548933</v>
+        <v>0.03600000425292382</v>
       </c>
       <c r="J35" s="8" t="n">
-        <v>0.04061250356615579</v>
+        <v>0.03910800426568259</v>
       </c>
       <c r="K35" s="3" t="n">
         <v>0</v>

</xml_diff>